<commit_message>
Deploy Sun 07/19/2026 13:29:39.57
</commit_message>
<xml_diff>
--- a/vertalis peptides/cenovnik.xlsx
+++ b/vertalis peptides/cenovnik.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\vertalis peptides\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\vertalis\vertalis peptides\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35EC940-BF54-43E3-856D-64F68F8858A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D36C6DA-C3E6-449F-BB86-95E61B1633AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2370" yWindow="2505" windowWidth="28725" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2370" yWindow="2505" windowWidth="28725" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Upload" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Deploy Sun 07/19/2026 16:15:01.01
</commit_message>
<xml_diff>
--- a/vertalis peptides/cenovnik.xlsx
+++ b/vertalis peptides/cenovnik.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\vertalis\vertalis peptides\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D36C6DA-C3E6-449F-BB86-95E61B1633AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AFABE76-5A80-4931-969C-68D8E6E4FA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2370" yWindow="2505" windowWidth="28725" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="2370" yWindow="2505" windowWidth="28725" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Upload" sheetId="1" r:id="rId1"/>
@@ -814,75 +814,75 @@
         <v>39.99</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="6">
         <v>3.8500000000000005</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="7">
         <v>15</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="6">
         <f t="shared" si="0"/>
         <v>31.992000000000004</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="7">
         <v>39.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="6">
         <v>6.6000000000000005</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="7">
         <v>25</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="6">
         <f t="shared" si="0"/>
         <v>51.991999999999997</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="7">
         <v>64.989999999999995</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="6">
         <v>8.8000000000000007</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="7">
         <v>40</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="6">
         <f t="shared" si="0"/>
         <v>47.992000000000004</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="7">
         <v>59.99</v>
       </c>
     </row>

</xml_diff>